<commit_message>
Apply metadata-only sample filtering
</commit_message>
<xml_diff>
--- a/all_QC_metadata.xlsx
+++ b/all_QC_metadata.xlsx
@@ -633,14 +633,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A94FB98-05C3-45B1-ACDE-C1CE92AA44E0}">
-  <dimension ref="A1:F28"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{8A94FB98-05C3-45B1-ACDE-C1CE92AA44E0}">
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultRowHeight="14" ns3:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17.08203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ns3:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>6</v>
       </c>
@@ -660,7 +660,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ns3:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
@@ -680,7 +680,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ns3:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
@@ -700,7 +700,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ns3:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -720,7 +720,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ns3:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -740,7 +740,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ns3:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>16</v>
       </c>
@@ -760,7 +760,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ns3:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
@@ -780,7 +780,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ns3:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>20</v>
       </c>
@@ -800,7 +800,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ns3:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>21</v>
       </c>
@@ -820,7 +820,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ns3:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -840,7 +840,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ns3:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
@@ -860,7 +860,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ns3:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>24</v>
       </c>
@@ -880,7 +880,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ns3:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>25</v>
       </c>
@@ -900,7 +900,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ns3:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>26</v>
       </c>
@@ -920,7 +920,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ns3:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>27</v>
       </c>
@@ -940,7 +940,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ns3:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>28</v>
       </c>
@@ -960,7 +960,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ns3:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>29</v>
       </c>
@@ -980,7 +980,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" ns3:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>30</v>
       </c>
@@ -1000,7 +1000,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ns3:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>31</v>
       </c>
@@ -1020,7 +1020,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ns3:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>32</v>
       </c>
@@ -1040,7 +1040,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ns3:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>33</v>
       </c>
@@ -1060,7 +1060,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ns3:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>34</v>
       </c>
@@ -1078,126 +1078,6 @@
       </c>
       <c r="F22" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C23" s="4">
-        <v>1</v>
-      </c>
-      <c r="D23" s="4">
-        <v>1</v>
-      </c>
-      <c r="E23" t="s">
-        <v>5</v>
-      </c>
-      <c r="F23" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C24" s="4">
-        <v>1</v>
-      </c>
-      <c r="D24" s="4">
-        <v>1</v>
-      </c>
-      <c r="E24" t="s">
-        <v>5</v>
-      </c>
-      <c r="F24" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" s="4">
-        <v>2</v>
-      </c>
-      <c r="D25" s="4">
-        <v>2</v>
-      </c>
-      <c r="E25" t="s">
-        <v>5</v>
-      </c>
-      <c r="F25" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C26" s="4">
-        <v>2</v>
-      </c>
-      <c r="D26" s="4">
-        <v>2</v>
-      </c>
-      <c r="E26" t="s">
-        <v>5</v>
-      </c>
-      <c r="F26" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C27" s="4">
-        <v>3</v>
-      </c>
-      <c r="D27" s="4">
-        <v>3</v>
-      </c>
-      <c r="E27" t="s">
-        <v>5</v>
-      </c>
-      <c r="F27" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C28" s="4">
-        <v>3</v>
-      </c>
-      <c r="D28" s="4">
-        <v>3</v>
-      </c>
-      <c r="E28" t="s">
-        <v>5</v>
-      </c>
-      <c r="F28" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clean sample columns using study and non-Blank QC metadata
* Add reproducible metadata-only sample filtering

* Apply metadata-only sample filtering

---------

Co-authored-by: github-actions[bot] <41898282+github-actions[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/all_QC_metadata.xlsx
+++ b/all_QC_metadata.xlsx
@@ -633,14 +633,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A94FB98-05C3-45B1-ACDE-C1CE92AA44E0}">
-  <dimension ref="A1:F28"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{8A94FB98-05C3-45B1-ACDE-C1CE92AA44E0}">
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultRowHeight="14" ns3:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17.08203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ns3:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>6</v>
       </c>
@@ -660,7 +660,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ns3:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
@@ -680,7 +680,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ns3:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
@@ -700,7 +700,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ns3:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -720,7 +720,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ns3:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -740,7 +740,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ns3:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>16</v>
       </c>
@@ -760,7 +760,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ns3:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
@@ -780,7 +780,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ns3:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>20</v>
       </c>
@@ -800,7 +800,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ns3:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>21</v>
       </c>
@@ -820,7 +820,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ns3:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -840,7 +840,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ns3:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
@@ -860,7 +860,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ns3:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>24</v>
       </c>
@@ -880,7 +880,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ns3:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>25</v>
       </c>
@@ -900,7 +900,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ns3:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>26</v>
       </c>
@@ -920,7 +920,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ns3:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>27</v>
       </c>
@@ -940,7 +940,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ns3:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>28</v>
       </c>
@@ -960,7 +960,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ns3:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>29</v>
       </c>
@@ -980,7 +980,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" ns3:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>30</v>
       </c>
@@ -1000,7 +1000,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ns3:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>31</v>
       </c>
@@ -1020,7 +1020,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ns3:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>32</v>
       </c>
@@ -1040,7 +1040,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ns3:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>33</v>
       </c>
@@ -1060,7 +1060,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ns3:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>34</v>
       </c>
@@ -1078,126 +1078,6 @@
       </c>
       <c r="F22" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C23" s="4">
-        <v>1</v>
-      </c>
-      <c r="D23" s="4">
-        <v>1</v>
-      </c>
-      <c r="E23" t="s">
-        <v>5</v>
-      </c>
-      <c r="F23" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C24" s="4">
-        <v>1</v>
-      </c>
-      <c r="D24" s="4">
-        <v>1</v>
-      </c>
-      <c r="E24" t="s">
-        <v>5</v>
-      </c>
-      <c r="F24" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" s="4">
-        <v>2</v>
-      </c>
-      <c r="D25" s="4">
-        <v>2</v>
-      </c>
-      <c r="E25" t="s">
-        <v>5</v>
-      </c>
-      <c r="F25" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C26" s="4">
-        <v>2</v>
-      </c>
-      <c r="D26" s="4">
-        <v>2</v>
-      </c>
-      <c r="E26" t="s">
-        <v>5</v>
-      </c>
-      <c r="F26" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C27" s="4">
-        <v>3</v>
-      </c>
-      <c r="D27" s="4">
-        <v>3</v>
-      </c>
-      <c r="E27" t="s">
-        <v>5</v>
-      </c>
-      <c r="F27" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C28" s="4">
-        <v>3</v>
-      </c>
-      <c r="D28" s="4">
-        <v>3</v>
-      </c>
-      <c r="E28" t="s">
-        <v>5</v>
-      </c>
-      <c r="F28" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>